<commit_message>
feat(modeles): ajout onglets PK_Coordonnees et OFFSETS_TRANSVERSAUX aux 4 modèles assainissement
Chaque fichier Excel dispose maintenant de deux nouveaux onglets :
- PK_Coordonnees : coordonnées Lambert 93 (X, Y, Z) + gisement + distance cumulée pour chaque PK
- OFFSETS_TRANSVERSAUX : distances transversales depuis l'axe par élément (G négatif / D positif)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/modeles_recepta/P1_RN_2x2voies_TPC_3km.xlsx
+++ b/data/modeles_recepta/P1_RN_2x2voies_TPC_3km.xlsx
@@ -1,25 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cote_Gauche" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cote_Droit" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGENDE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cote_Gauche" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cote_Droit" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="LEGENDE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PK_Coordonnees" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="OFFSETS_TRANSVERSAUX" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PK_Coordonnees'!$A$3:$F$125</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="9">
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="#,##0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="+0.000;-0.000;0.000"/>
+  </numFmts>
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +72,77 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00475569"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001E293B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <b val="1"/>
+      <color rgb="000F4C35"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <color rgb="00475569"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F766E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F766E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -135,8 +214,58 @@
         <fgColor rgb="000D1F38"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFBEB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F4C35"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDF4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0FFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -158,11 +287,25 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -239,6 +382,87 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="14" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="14" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -313,36 +537,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="9334500" cy="3429000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14610,6 +14804,3161 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F127"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>COORDONNÉES DE L'AXE — Route Nationale 2x2 voies TPC — 3 km</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Système de référence : Lambert 93 (EPSG:2154)  —  Données à renseigner avec les coordonnées réelles du levé</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>X (m)</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>Y (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>Z axe (m)</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>Gisement (°)</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>Dist. cumulée (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Point kilométrique</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>Lambert 93 — Est</t>
+        </is>
+      </c>
+      <c r="C4" s="29" t="inlineStr">
+        <is>
+          <t>Lambert 93 — Nord</t>
+        </is>
+      </c>
+      <c r="D4" s="29" t="inlineStr">
+        <is>
+          <t>Cote NGF de l'axe chaussée</t>
+        </is>
+      </c>
+      <c r="E4" s="29" t="inlineStr">
+        <is>
+          <t>Direction route (0°=N, 90°=E)</t>
+        </is>
+      </c>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t>Distance depuis l'origine</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>0+000</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="n">
+        <v>839420</v>
+      </c>
+      <c r="C5" s="31" t="n">
+        <v>6516800</v>
+      </c>
+      <c r="D5" s="32" t="n">
+        <v>105.85</v>
+      </c>
+      <c r="E5" s="33" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="F5" s="34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>0+025</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n">
+        <v>839436.92</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <v>6516818.404</v>
+      </c>
+      <c r="D6" s="37" t="n">
+        <v>105.887</v>
+      </c>
+      <c r="E6" s="38" t="n">
+        <v>42.5937</v>
+      </c>
+      <c r="F6" s="39" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>0+050</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="n">
+        <v>839453.9</v>
+      </c>
+      <c r="C7" s="36" t="n">
+        <v>6516836.753</v>
+      </c>
+      <c r="D7" s="37" t="n">
+        <v>105.925</v>
+      </c>
+      <c r="E7" s="38" t="n">
+        <v>42.6874</v>
+      </c>
+      <c r="F7" s="39" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>0+075</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>839470.9399999999</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>6516855.047</v>
+      </c>
+      <c r="D8" s="37" t="n">
+        <v>105.962</v>
+      </c>
+      <c r="E8" s="38" t="n">
+        <v>42.7808</v>
+      </c>
+      <c r="F8" s="39" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>0+100</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="n">
+        <v>839488.039</v>
+      </c>
+      <c r="C9" s="31" t="n">
+        <v>6516873.285</v>
+      </c>
+      <c r="D9" s="32" t="n">
+        <v>106</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <v>42.874</v>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>0+125</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>839505.197</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>6516891.469</v>
+      </c>
+      <c r="D10" s="37" t="n">
+        <v>106.037</v>
+      </c>
+      <c r="E10" s="38" t="n">
+        <v>42.9668</v>
+      </c>
+      <c r="F10" s="39" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>0+150</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>839522.4129999999</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>6516909.597</v>
+      </c>
+      <c r="D11" s="37" t="n">
+        <v>106.075</v>
+      </c>
+      <c r="E11" s="38" t="n">
+        <v>43.0592</v>
+      </c>
+      <c r="F11" s="39" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>0+175</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="n">
+        <v>839539.687</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>6516927.672</v>
+      </c>
+      <c r="D12" s="37" t="n">
+        <v>106.112</v>
+      </c>
+      <c r="E12" s="38" t="n">
+        <v>43.151</v>
+      </c>
+      <c r="F12" s="39" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>0+200</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="n">
+        <v>839557.017</v>
+      </c>
+      <c r="C13" s="31" t="n">
+        <v>6516945.693</v>
+      </c>
+      <c r="D13" s="32" t="n">
+        <v>106.15</v>
+      </c>
+      <c r="E13" s="33" t="n">
+        <v>43.2422</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>0+225</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="n">
+        <v>839574.402</v>
+      </c>
+      <c r="C14" s="36" t="n">
+        <v>6516963.661</v>
+      </c>
+      <c r="D14" s="37" t="n">
+        <v>106.188</v>
+      </c>
+      <c r="E14" s="38" t="n">
+        <v>43.3327</v>
+      </c>
+      <c r="F14" s="39" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>0+250</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="n">
+        <v>839591.843</v>
+      </c>
+      <c r="C15" s="36" t="n">
+        <v>6516981.577</v>
+      </c>
+      <c r="D15" s="37" t="n">
+        <v>106.225</v>
+      </c>
+      <c r="E15" s="38" t="n">
+        <v>43.4223</v>
+      </c>
+      <c r="F15" s="39" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>0+275</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="n">
+        <v>839609.336</v>
+      </c>
+      <c r="C16" s="36" t="n">
+        <v>6516999.441</v>
+      </c>
+      <c r="D16" s="37" t="n">
+        <v>106.262</v>
+      </c>
+      <c r="E16" s="38" t="n">
+        <v>43.5111</v>
+      </c>
+      <c r="F16" s="39" t="n">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>0+300</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="n">
+        <v>839626.8810000001</v>
+      </c>
+      <c r="C17" s="31" t="n">
+        <v>6517017.256</v>
+      </c>
+      <c r="D17" s="32" t="n">
+        <v>106.3</v>
+      </c>
+      <c r="E17" s="33" t="n">
+        <v>43.5988</v>
+      </c>
+      <c r="F17" s="34" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>0+325</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="n">
+        <v>839644.477</v>
+      </c>
+      <c r="C18" s="36" t="n">
+        <v>6517035.021</v>
+      </c>
+      <c r="D18" s="37" t="n">
+        <v>106.337</v>
+      </c>
+      <c r="E18" s="38" t="n">
+        <v>43.6855</v>
+      </c>
+      <c r="F18" s="39" t="n">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>0+350</t>
+        </is>
+      </c>
+      <c r="B19" s="36" t="n">
+        <v>839662.122</v>
+      </c>
+      <c r="C19" s="36" t="n">
+        <v>6517052.739</v>
+      </c>
+      <c r="D19" s="37" t="n">
+        <v>106.375</v>
+      </c>
+      <c r="E19" s="38" t="n">
+        <v>43.771</v>
+      </c>
+      <c r="F19" s="39" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>0+375</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="n">
+        <v>839679.8149999999</v>
+      </c>
+      <c r="C20" s="36" t="n">
+        <v>6517070.409</v>
+      </c>
+      <c r="D20" s="37" t="n">
+        <v>106.412</v>
+      </c>
+      <c r="E20" s="38" t="n">
+        <v>43.8553</v>
+      </c>
+      <c r="F20" s="39" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>0+400</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="n">
+        <v>839697.553</v>
+      </c>
+      <c r="C21" s="31" t="n">
+        <v>6517088.035</v>
+      </c>
+      <c r="D21" s="32" t="n">
+        <v>106.45</v>
+      </c>
+      <c r="E21" s="33" t="n">
+        <v>43.9383</v>
+      </c>
+      <c r="F21" s="34" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>0+425</t>
+        </is>
+      </c>
+      <c r="B22" s="36" t="n">
+        <v>839715.336</v>
+      </c>
+      <c r="C22" s="36" t="n">
+        <v>6517105.617</v>
+      </c>
+      <c r="D22" s="37" t="n">
+        <v>106.487</v>
+      </c>
+      <c r="E22" s="38" t="n">
+        <v>44.0198</v>
+      </c>
+      <c r="F22" s="39" t="n">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="35" t="inlineStr">
+        <is>
+          <t>0+450</t>
+        </is>
+      </c>
+      <c r="B23" s="36" t="n">
+        <v>839733.16</v>
+      </c>
+      <c r="C23" s="36" t="n">
+        <v>6517123.157</v>
+      </c>
+      <c r="D23" s="37" t="n">
+        <v>106.525</v>
+      </c>
+      <c r="E23" s="38" t="n">
+        <v>44.0999</v>
+      </c>
+      <c r="F23" s="39" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>0+475</t>
+        </is>
+      </c>
+      <c r="B24" s="36" t="n">
+        <v>839751.025</v>
+      </c>
+      <c r="C24" s="36" t="n">
+        <v>6517140.657</v>
+      </c>
+      <c r="D24" s="37" t="n">
+        <v>106.562</v>
+      </c>
+      <c r="E24" s="38" t="n">
+        <v>44.1784</v>
+      </c>
+      <c r="F24" s="39" t="n">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>0+500</t>
+        </is>
+      </c>
+      <c r="B25" s="31" t="n">
+        <v>839768.928</v>
+      </c>
+      <c r="C25" s="31" t="n">
+        <v>6517158.119</v>
+      </c>
+      <c r="D25" s="32" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="E25" s="33" t="n">
+        <v>44.2553</v>
+      </c>
+      <c r="F25" s="34" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="35" t="inlineStr">
+        <is>
+          <t>0+525</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="n">
+        <v>839786.868</v>
+      </c>
+      <c r="C26" s="36" t="n">
+        <v>6517175.544</v>
+      </c>
+      <c r="D26" s="37" t="n">
+        <v>106.637</v>
+      </c>
+      <c r="E26" s="38" t="n">
+        <v>44.3305</v>
+      </c>
+      <c r="F26" s="39" t="n">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="35" t="inlineStr">
+        <is>
+          <t>0+550</t>
+        </is>
+      </c>
+      <c r="B27" s="36" t="n">
+        <v>839804.841</v>
+      </c>
+      <c r="C27" s="36" t="n">
+        <v>6517192.934</v>
+      </c>
+      <c r="D27" s="37" t="n">
+        <v>106.675</v>
+      </c>
+      <c r="E27" s="38" t="n">
+        <v>44.4038</v>
+      </c>
+      <c r="F27" s="39" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="35" t="inlineStr">
+        <is>
+          <t>0+575</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="n">
+        <v>839822.846</v>
+      </c>
+      <c r="C28" s="36" t="n">
+        <v>6517210.292</v>
+      </c>
+      <c r="D28" s="37" t="n">
+        <v>106.712</v>
+      </c>
+      <c r="E28" s="38" t="n">
+        <v>44.4753</v>
+      </c>
+      <c r="F28" s="39" t="n">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>0+600</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="n">
+        <v>839840.8810000001</v>
+      </c>
+      <c r="C29" s="31" t="n">
+        <v>6517227.62</v>
+      </c>
+      <c r="D29" s="32" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="E29" s="33" t="n">
+        <v>44.5449</v>
+      </c>
+      <c r="F29" s="34" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="35" t="inlineStr">
+        <is>
+          <t>0+625</t>
+        </is>
+      </c>
+      <c r="B30" s="36" t="n">
+        <v>839858.943</v>
+      </c>
+      <c r="C30" s="36" t="n">
+        <v>6517244.921</v>
+      </c>
+      <c r="D30" s="37" t="n">
+        <v>106.787</v>
+      </c>
+      <c r="E30" s="38" t="n">
+        <v>44.6125</v>
+      </c>
+      <c r="F30" s="39" t="n">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="35" t="inlineStr">
+        <is>
+          <t>0+650</t>
+        </is>
+      </c>
+      <c r="B31" s="36" t="n">
+        <v>839877.029</v>
+      </c>
+      <c r="C31" s="36" t="n">
+        <v>6517262.195</v>
+      </c>
+      <c r="D31" s="37" t="n">
+        <v>106.825</v>
+      </c>
+      <c r="E31" s="38" t="n">
+        <v>44.678</v>
+      </c>
+      <c r="F31" s="39" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="35" t="inlineStr">
+        <is>
+          <t>0+675</t>
+        </is>
+      </c>
+      <c r="B32" s="36" t="n">
+        <v>839895.138</v>
+      </c>
+      <c r="C32" s="36" t="n">
+        <v>6517279.446</v>
+      </c>
+      <c r="D32" s="37" t="n">
+        <v>106.862</v>
+      </c>
+      <c r="E32" s="38" t="n">
+        <v>44.7414</v>
+      </c>
+      <c r="F32" s="39" t="n">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>0+700</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="n">
+        <v>839913.267</v>
+      </c>
+      <c r="C33" s="31" t="n">
+        <v>6517296.677</v>
+      </c>
+      <c r="D33" s="32" t="n">
+        <v>106.9</v>
+      </c>
+      <c r="E33" s="33" t="n">
+        <v>44.8026</v>
+      </c>
+      <c r="F33" s="34" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="35" t="inlineStr">
+        <is>
+          <t>0+725</t>
+        </is>
+      </c>
+      <c r="B34" s="36" t="n">
+        <v>839931.4129999999</v>
+      </c>
+      <c r="C34" s="36" t="n">
+        <v>6517313.889</v>
+      </c>
+      <c r="D34" s="37" t="n">
+        <v>106.938</v>
+      </c>
+      <c r="E34" s="38" t="n">
+        <v>44.8616</v>
+      </c>
+      <c r="F34" s="39" t="n">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="35" t="inlineStr">
+        <is>
+          <t>0+750</t>
+        </is>
+      </c>
+      <c r="B35" s="36" t="n">
+        <v>839949.573</v>
+      </c>
+      <c r="C35" s="36" t="n">
+        <v>6517331.086</v>
+      </c>
+      <c r="D35" s="37" t="n">
+        <v>106.975</v>
+      </c>
+      <c r="E35" s="38" t="n">
+        <v>44.9182</v>
+      </c>
+      <c r="F35" s="39" t="n">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="35" t="inlineStr">
+        <is>
+          <t>0+775</t>
+        </is>
+      </c>
+      <c r="B36" s="36" t="n">
+        <v>839967.745</v>
+      </c>
+      <c r="C36" s="36" t="n">
+        <v>6517348.27</v>
+      </c>
+      <c r="D36" s="37" t="n">
+        <v>107.012</v>
+      </c>
+      <c r="E36" s="38" t="n">
+        <v>44.9725</v>
+      </c>
+      <c r="F36" s="39" t="n">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
+          <t>0+800</t>
+        </is>
+      </c>
+      <c r="B37" s="31" t="n">
+        <v>839985.926</v>
+      </c>
+      <c r="C37" s="31" t="n">
+        <v>6517365.444</v>
+      </c>
+      <c r="D37" s="32" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="E37" s="33" t="n">
+        <v>45.0244</v>
+      </c>
+      <c r="F37" s="34" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="35" t="inlineStr">
+        <is>
+          <t>0+825</t>
+        </is>
+      </c>
+      <c r="B38" s="36" t="n">
+        <v>840004.1139999999</v>
+      </c>
+      <c r="C38" s="36" t="n">
+        <v>6517382.611</v>
+      </c>
+      <c r="D38" s="37" t="n">
+        <v>107.087</v>
+      </c>
+      <c r="E38" s="38" t="n">
+        <v>45.0738</v>
+      </c>
+      <c r="F38" s="39" t="n">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>0+850</t>
+        </is>
+      </c>
+      <c r="B39" s="36" t="n">
+        <v>840022.306</v>
+      </c>
+      <c r="C39" s="36" t="n">
+        <v>6517399.773</v>
+      </c>
+      <c r="D39" s="37" t="n">
+        <v>107.125</v>
+      </c>
+      <c r="E39" s="38" t="n">
+        <v>45.1207</v>
+      </c>
+      <c r="F39" s="39" t="n">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="35" t="inlineStr">
+        <is>
+          <t>0+875</t>
+        </is>
+      </c>
+      <c r="B40" s="36" t="n">
+        <v>840040.498</v>
+      </c>
+      <c r="C40" s="36" t="n">
+        <v>6517416.933</v>
+      </c>
+      <c r="D40" s="37" t="n">
+        <v>107.162</v>
+      </c>
+      <c r="E40" s="38" t="n">
+        <v>45.1651</v>
+      </c>
+      <c r="F40" s="39" t="n">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>0+900</t>
+        </is>
+      </c>
+      <c r="B41" s="31" t="n">
+        <v>840058.689</v>
+      </c>
+      <c r="C41" s="31" t="n">
+        <v>6517434.095</v>
+      </c>
+      <c r="D41" s="32" t="n">
+        <v>107.2</v>
+      </c>
+      <c r="E41" s="33" t="n">
+        <v>45.2068</v>
+      </c>
+      <c r="F41" s="34" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="35" t="inlineStr">
+        <is>
+          <t>0+925</t>
+        </is>
+      </c>
+      <c r="B42" s="36" t="n">
+        <v>840076.875</v>
+      </c>
+      <c r="C42" s="36" t="n">
+        <v>6517451.261</v>
+      </c>
+      <c r="D42" s="37" t="n">
+        <v>107.237</v>
+      </c>
+      <c r="E42" s="38" t="n">
+        <v>45.2459</v>
+      </c>
+      <c r="F42" s="39" t="n">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="35" t="inlineStr">
+        <is>
+          <t>0+950</t>
+        </is>
+      </c>
+      <c r="B43" s="36" t="n">
+        <v>840095.053</v>
+      </c>
+      <c r="C43" s="36" t="n">
+        <v>6517468.433</v>
+      </c>
+      <c r="D43" s="37" t="n">
+        <v>107.275</v>
+      </c>
+      <c r="E43" s="38" t="n">
+        <v>45.2823</v>
+      </c>
+      <c r="F43" s="39" t="n">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="35" t="inlineStr">
+        <is>
+          <t>0+975</t>
+        </is>
+      </c>
+      <c r="B44" s="36" t="n">
+        <v>840113.221</v>
+      </c>
+      <c r="C44" s="36" t="n">
+        <v>6517485.616</v>
+      </c>
+      <c r="D44" s="37" t="n">
+        <v>107.312</v>
+      </c>
+      <c r="E44" s="38" t="n">
+        <v>45.316</v>
+      </c>
+      <c r="F44" s="39" t="n">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>1+000</t>
+        </is>
+      </c>
+      <c r="B45" s="31" t="n">
+        <v>840131.376</v>
+      </c>
+      <c r="C45" s="31" t="n">
+        <v>6517502.812</v>
+      </c>
+      <c r="D45" s="32" t="n">
+        <v>107.35</v>
+      </c>
+      <c r="E45" s="33" t="n">
+        <v>45.347</v>
+      </c>
+      <c r="F45" s="34" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="35" t="inlineStr">
+        <is>
+          <t>1+025</t>
+        </is>
+      </c>
+      <c r="B46" s="36" t="n">
+        <v>840149.514</v>
+      </c>
+      <c r="C46" s="36" t="n">
+        <v>6517520.024</v>
+      </c>
+      <c r="D46" s="37" t="n">
+        <v>107.387</v>
+      </c>
+      <c r="E46" s="38" t="n">
+        <v>45.3751</v>
+      </c>
+      <c r="F46" s="39" t="n">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="35" t="inlineStr">
+        <is>
+          <t>1+050</t>
+        </is>
+      </c>
+      <c r="B47" s="36" t="n">
+        <v>840167.634</v>
+      </c>
+      <c r="C47" s="36" t="n">
+        <v>6517537.254</v>
+      </c>
+      <c r="D47" s="37" t="n">
+        <v>107.425</v>
+      </c>
+      <c r="E47" s="38" t="n">
+        <v>45.4005</v>
+      </c>
+      <c r="F47" s="39" t="n">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="35" t="inlineStr">
+        <is>
+          <t>1+075</t>
+        </is>
+      </c>
+      <c r="B48" s="36" t="n">
+        <v>840185.731</v>
+      </c>
+      <c r="C48" s="36" t="n">
+        <v>6517554.507</v>
+      </c>
+      <c r="D48" s="37" t="n">
+        <v>107.462</v>
+      </c>
+      <c r="E48" s="38" t="n">
+        <v>45.423</v>
+      </c>
+      <c r="F48" s="39" t="n">
+        <v>1075</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="30" t="inlineStr">
+        <is>
+          <t>1+100</t>
+        </is>
+      </c>
+      <c r="B49" s="31" t="n">
+        <v>840203.804</v>
+      </c>
+      <c r="C49" s="31" t="n">
+        <v>6517571.785</v>
+      </c>
+      <c r="D49" s="32" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="E49" s="33" t="n">
+        <v>45.4427</v>
+      </c>
+      <c r="F49" s="34" t="n">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="35" t="inlineStr">
+        <is>
+          <t>1+125</t>
+        </is>
+      </c>
+      <c r="B50" s="36" t="n">
+        <v>840221.849</v>
+      </c>
+      <c r="C50" s="36" t="n">
+        <v>6517589.09</v>
+      </c>
+      <c r="D50" s="37" t="n">
+        <v>107.537</v>
+      </c>
+      <c r="E50" s="38" t="n">
+        <v>45.4595</v>
+      </c>
+      <c r="F50" s="39" t="n">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="35" t="inlineStr">
+        <is>
+          <t>1+150</t>
+        </is>
+      </c>
+      <c r="B51" s="36" t="n">
+        <v>840239.8639999999</v>
+      </c>
+      <c r="C51" s="36" t="n">
+        <v>6517606.427</v>
+      </c>
+      <c r="D51" s="37" t="n">
+        <v>107.575</v>
+      </c>
+      <c r="E51" s="38" t="n">
+        <v>45.4734</v>
+      </c>
+      <c r="F51" s="39" t="n">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="35" t="inlineStr">
+        <is>
+          <t>1+175</t>
+        </is>
+      </c>
+      <c r="B52" s="36" t="n">
+        <v>840257.845</v>
+      </c>
+      <c r="C52" s="36" t="n">
+        <v>6517623.797</v>
+      </c>
+      <c r="D52" s="37" t="n">
+        <v>107.612</v>
+      </c>
+      <c r="E52" s="38" t="n">
+        <v>45.4844</v>
+      </c>
+      <c r="F52" s="39" t="n">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="30" t="inlineStr">
+        <is>
+          <t>1+200</t>
+        </is>
+      </c>
+      <c r="B53" s="31" t="n">
+        <v>840275.79</v>
+      </c>
+      <c r="C53" s="31" t="n">
+        <v>6517641.203</v>
+      </c>
+      <c r="D53" s="32" t="n">
+        <v>107.65</v>
+      </c>
+      <c r="E53" s="33" t="n">
+        <v>45.4925</v>
+      </c>
+      <c r="F53" s="34" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="35" t="inlineStr">
+        <is>
+          <t>1+225</t>
+        </is>
+      </c>
+      <c r="B54" s="36" t="n">
+        <v>840293.697</v>
+      </c>
+      <c r="C54" s="36" t="n">
+        <v>6517658.65</v>
+      </c>
+      <c r="D54" s="37" t="n">
+        <v>107.688</v>
+      </c>
+      <c r="E54" s="38" t="n">
+        <v>45.4977</v>
+      </c>
+      <c r="F54" s="39" t="n">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="35" t="inlineStr">
+        <is>
+          <t>1+250</t>
+        </is>
+      </c>
+      <c r="B55" s="36" t="n">
+        <v>840311.561</v>
+      </c>
+      <c r="C55" s="36" t="n">
+        <v>6517676.138</v>
+      </c>
+      <c r="D55" s="37" t="n">
+        <v>107.725</v>
+      </c>
+      <c r="E55" s="38" t="n">
+        <v>45.4999</v>
+      </c>
+      <c r="F55" s="39" t="n">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="35" t="inlineStr">
+        <is>
+          <t>1+275</t>
+        </is>
+      </c>
+      <c r="B56" s="36" t="n">
+        <v>840329.382</v>
+      </c>
+      <c r="C56" s="36" t="n">
+        <v>6517693.672</v>
+      </c>
+      <c r="D56" s="37" t="n">
+        <v>107.762</v>
+      </c>
+      <c r="E56" s="38" t="n">
+        <v>45.4992</v>
+      </c>
+      <c r="F56" s="39" t="n">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="30" t="inlineStr">
+        <is>
+          <t>1+300</t>
+        </is>
+      </c>
+      <c r="B57" s="31" t="n">
+        <v>840347.156</v>
+      </c>
+      <c r="C57" s="31" t="n">
+        <v>6517711.253</v>
+      </c>
+      <c r="D57" s="32" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="E57" s="33" t="n">
+        <v>45.4956</v>
+      </c>
+      <c r="F57" s="34" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="35" t="inlineStr">
+        <is>
+          <t>1+325</t>
+        </is>
+      </c>
+      <c r="B58" s="36" t="n">
+        <v>840364.879</v>
+      </c>
+      <c r="C58" s="36" t="n">
+        <v>6517728.885</v>
+      </c>
+      <c r="D58" s="37" t="n">
+        <v>107.837</v>
+      </c>
+      <c r="E58" s="38" t="n">
+        <v>45.4891</v>
+      </c>
+      <c r="F58" s="39" t="n">
+        <v>1325</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="35" t="inlineStr">
+        <is>
+          <t>1+350</t>
+        </is>
+      </c>
+      <c r="B59" s="36" t="n">
+        <v>840382.551</v>
+      </c>
+      <c r="C59" s="36" t="n">
+        <v>6517746.57</v>
+      </c>
+      <c r="D59" s="37" t="n">
+        <v>107.875</v>
+      </c>
+      <c r="E59" s="38" t="n">
+        <v>45.4796</v>
+      </c>
+      <c r="F59" s="39" t="n">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="35" t="inlineStr">
+        <is>
+          <t>1+375</t>
+        </is>
+      </c>
+      <c r="B60" s="36" t="n">
+        <v>840400.1679999999</v>
+      </c>
+      <c r="C60" s="36" t="n">
+        <v>6517764.311</v>
+      </c>
+      <c r="D60" s="37" t="n">
+        <v>107.912</v>
+      </c>
+      <c r="E60" s="38" t="n">
+        <v>45.4672</v>
+      </c>
+      <c r="F60" s="39" t="n">
+        <v>1375</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="30" t="inlineStr">
+        <is>
+          <t>1+400</t>
+        </is>
+      </c>
+      <c r="B61" s="31" t="n">
+        <v>840417.727</v>
+      </c>
+      <c r="C61" s="31" t="n">
+        <v>6517782.11</v>
+      </c>
+      <c r="D61" s="32" t="n">
+        <v>107.95</v>
+      </c>
+      <c r="E61" s="33" t="n">
+        <v>45.452</v>
+      </c>
+      <c r="F61" s="34" t="n">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="35" t="inlineStr">
+        <is>
+          <t>1+425</t>
+        </is>
+      </c>
+      <c r="B62" s="36" t="n">
+        <v>840435.227</v>
+      </c>
+      <c r="C62" s="36" t="n">
+        <v>6517799.969</v>
+      </c>
+      <c r="D62" s="37" t="n">
+        <v>107.987</v>
+      </c>
+      <c r="E62" s="38" t="n">
+        <v>45.4338</v>
+      </c>
+      <c r="F62" s="39" t="n">
+        <v>1425</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="35" t="inlineStr">
+        <is>
+          <t>1+450</t>
+        </is>
+      </c>
+      <c r="B63" s="36" t="n">
+        <v>840452.665</v>
+      </c>
+      <c r="C63" s="36" t="n">
+        <v>6517817.891</v>
+      </c>
+      <c r="D63" s="37" t="n">
+        <v>108.025</v>
+      </c>
+      <c r="E63" s="38" t="n">
+        <v>45.4128</v>
+      </c>
+      <c r="F63" s="39" t="n">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="35" t="inlineStr">
+        <is>
+          <t>1+475</t>
+        </is>
+      </c>
+      <c r="B64" s="36" t="n">
+        <v>840470.0379999999</v>
+      </c>
+      <c r="C64" s="36" t="n">
+        <v>6517835.879</v>
+      </c>
+      <c r="D64" s="37" t="n">
+        <v>108.062</v>
+      </c>
+      <c r="E64" s="38" t="n">
+        <v>45.3889</v>
+      </c>
+      <c r="F64" s="39" t="n">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="30" t="inlineStr">
+        <is>
+          <t>1+500</t>
+        </is>
+      </c>
+      <c r="B65" s="31" t="n">
+        <v>840487.345</v>
+      </c>
+      <c r="C65" s="31" t="n">
+        <v>6517853.933</v>
+      </c>
+      <c r="D65" s="32" t="n">
+        <v>108.1</v>
+      </c>
+      <c r="E65" s="33" t="n">
+        <v>45.3623</v>
+      </c>
+      <c r="F65" s="34" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="35" t="inlineStr">
+        <is>
+          <t>1+525</t>
+        </is>
+      </c>
+      <c r="B66" s="36" t="n">
+        <v>840504.583</v>
+      </c>
+      <c r="C66" s="36" t="n">
+        <v>6517872.057</v>
+      </c>
+      <c r="D66" s="37" t="n">
+        <v>108.137</v>
+      </c>
+      <c r="E66" s="38" t="n">
+        <v>45.3328</v>
+      </c>
+      <c r="F66" s="39" t="n">
+        <v>1525</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="35" t="inlineStr">
+        <is>
+          <t>1+550</t>
+        </is>
+      </c>
+      <c r="B67" s="36" t="n">
+        <v>840521.75</v>
+      </c>
+      <c r="C67" s="36" t="n">
+        <v>6517890.251</v>
+      </c>
+      <c r="D67" s="37" t="n">
+        <v>108.175</v>
+      </c>
+      <c r="E67" s="38" t="n">
+        <v>45.3005</v>
+      </c>
+      <c r="F67" s="39" t="n">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="35" t="inlineStr">
+        <is>
+          <t>1+575</t>
+        </is>
+      </c>
+      <c r="B68" s="36" t="n">
+        <v>840538.843</v>
+      </c>
+      <c r="C68" s="36" t="n">
+        <v>6517908.519</v>
+      </c>
+      <c r="D68" s="37" t="n">
+        <v>108.212</v>
+      </c>
+      <c r="E68" s="38" t="n">
+        <v>45.2656</v>
+      </c>
+      <c r="F68" s="39" t="n">
+        <v>1575</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="30" t="inlineStr">
+        <is>
+          <t>1+600</t>
+        </is>
+      </c>
+      <c r="B69" s="31" t="n">
+        <v>840555.862</v>
+      </c>
+      <c r="C69" s="31" t="n">
+        <v>6517926.862</v>
+      </c>
+      <c r="D69" s="32" t="n">
+        <v>108.25</v>
+      </c>
+      <c r="E69" s="33" t="n">
+        <v>45.2279</v>
+      </c>
+      <c r="F69" s="34" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="35" t="inlineStr">
+        <is>
+          <t>1+625</t>
+        </is>
+      </c>
+      <c r="B70" s="36" t="n">
+        <v>840572.804</v>
+      </c>
+      <c r="C70" s="36" t="n">
+        <v>6517945.281</v>
+      </c>
+      <c r="D70" s="37" t="n">
+        <v>108.287</v>
+      </c>
+      <c r="E70" s="38" t="n">
+        <v>45.1876</v>
+      </c>
+      <c r="F70" s="39" t="n">
+        <v>1625</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="35" t="inlineStr">
+        <is>
+          <t>1+650</t>
+        </is>
+      </c>
+      <c r="B71" s="36" t="n">
+        <v>840589.667</v>
+      </c>
+      <c r="C71" s="36" t="n">
+        <v>6517963.778</v>
+      </c>
+      <c r="D71" s="37" t="n">
+        <v>108.325</v>
+      </c>
+      <c r="E71" s="38" t="n">
+        <v>45.1446</v>
+      </c>
+      <c r="F71" s="39" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="35" t="inlineStr">
+        <is>
+          <t>1+675</t>
+        </is>
+      </c>
+      <c r="B72" s="36" t="n">
+        <v>840606.449</v>
+      </c>
+      <c r="C72" s="36" t="n">
+        <v>6517982.355</v>
+      </c>
+      <c r="D72" s="37" t="n">
+        <v>108.362</v>
+      </c>
+      <c r="E72" s="38" t="n">
+        <v>45.099</v>
+      </c>
+      <c r="F72" s="39" t="n">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="30" t="inlineStr">
+        <is>
+          <t>1+700</t>
+        </is>
+      </c>
+      <c r="B73" s="31" t="n">
+        <v>840623.15</v>
+      </c>
+      <c r="C73" s="31" t="n">
+        <v>6518001.012</v>
+      </c>
+      <c r="D73" s="32" t="n">
+        <v>108.4</v>
+      </c>
+      <c r="E73" s="33" t="n">
+        <v>45.051</v>
+      </c>
+      <c r="F73" s="34" t="n">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="35" t="inlineStr">
+        <is>
+          <t>1+725</t>
+        </is>
+      </c>
+      <c r="B74" s="36" t="n">
+        <v>840639.767</v>
+      </c>
+      <c r="C74" s="36" t="n">
+        <v>6518019.751</v>
+      </c>
+      <c r="D74" s="37" t="n">
+        <v>108.438</v>
+      </c>
+      <c r="E74" s="38" t="n">
+        <v>45.0004</v>
+      </c>
+      <c r="F74" s="39" t="n">
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="35" t="inlineStr">
+        <is>
+          <t>1+750</t>
+        </is>
+      </c>
+      <c r="B75" s="36" t="n">
+        <v>840656.3</v>
+      </c>
+      <c r="C75" s="36" t="n">
+        <v>6518038.573</v>
+      </c>
+      <c r="D75" s="37" t="n">
+        <v>108.475</v>
+      </c>
+      <c r="E75" s="38" t="n">
+        <v>44.9474</v>
+      </c>
+      <c r="F75" s="39" t="n">
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="35" t="inlineStr">
+        <is>
+          <t>1+775</t>
+        </is>
+      </c>
+      <c r="B76" s="36" t="n">
+        <v>840672.746</v>
+      </c>
+      <c r="C76" s="36" t="n">
+        <v>6518057.479</v>
+      </c>
+      <c r="D76" s="37" t="n">
+        <v>108.512</v>
+      </c>
+      <c r="E76" s="38" t="n">
+        <v>44.892</v>
+      </c>
+      <c r="F76" s="39" t="n">
+        <v>1775</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
+        <is>
+          <t>1+800</t>
+        </is>
+      </c>
+      <c r="B77" s="31" t="n">
+        <v>840689.1040000001</v>
+      </c>
+      <c r="C77" s="31" t="n">
+        <v>6518076.47</v>
+      </c>
+      <c r="D77" s="32" t="n">
+        <v>108.55</v>
+      </c>
+      <c r="E77" s="33" t="n">
+        <v>44.8342</v>
+      </c>
+      <c r="F77" s="34" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="35" t="inlineStr">
+        <is>
+          <t>1+825</t>
+        </is>
+      </c>
+      <c r="B78" s="36" t="n">
+        <v>840705.374</v>
+      </c>
+      <c r="C78" s="36" t="n">
+        <v>6518095.546</v>
+      </c>
+      <c r="D78" s="37" t="n">
+        <v>108.587</v>
+      </c>
+      <c r="E78" s="38" t="n">
+        <v>44.7742</v>
+      </c>
+      <c r="F78" s="39" t="n">
+        <v>1825</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="35" t="inlineStr">
+        <is>
+          <t>1+850</t>
+        </is>
+      </c>
+      <c r="B79" s="36" t="n">
+        <v>840721.5550000001</v>
+      </c>
+      <c r="C79" s="36" t="n">
+        <v>6518114.707</v>
+      </c>
+      <c r="D79" s="37" t="n">
+        <v>108.625</v>
+      </c>
+      <c r="E79" s="38" t="n">
+        <v>44.712</v>
+      </c>
+      <c r="F79" s="39" t="n">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="35" t="inlineStr">
+        <is>
+          <t>1+875</t>
+        </is>
+      </c>
+      <c r="B80" s="36" t="n">
+        <v>840737.645</v>
+      </c>
+      <c r="C80" s="36" t="n">
+        <v>6518133.956</v>
+      </c>
+      <c r="D80" s="37" t="n">
+        <v>108.662</v>
+      </c>
+      <c r="E80" s="38" t="n">
+        <v>44.6476</v>
+      </c>
+      <c r="F80" s="39" t="n">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="30" t="inlineStr">
+        <is>
+          <t>1+900</t>
+        </is>
+      </c>
+      <c r="B81" s="31" t="n">
+        <v>840753.643</v>
+      </c>
+      <c r="C81" s="31" t="n">
+        <v>6518153.291</v>
+      </c>
+      <c r="D81" s="32" t="n">
+        <v>108.7</v>
+      </c>
+      <c r="E81" s="33" t="n">
+        <v>44.5811</v>
+      </c>
+      <c r="F81" s="34" t="n">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="35" t="inlineStr">
+        <is>
+          <t>1+925</t>
+        </is>
+      </c>
+      <c r="B82" s="36" t="n">
+        <v>840769.55</v>
+      </c>
+      <c r="C82" s="36" t="n">
+        <v>6518172.712</v>
+      </c>
+      <c r="D82" s="37" t="n">
+        <v>108.737</v>
+      </c>
+      <c r="E82" s="38" t="n">
+        <v>44.5125</v>
+      </c>
+      <c r="F82" s="39" t="n">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="35" t="inlineStr">
+        <is>
+          <t>1+950</t>
+        </is>
+      </c>
+      <c r="B83" s="36" t="n">
+        <v>840785.365</v>
+      </c>
+      <c r="C83" s="36" t="n">
+        <v>6518192.221</v>
+      </c>
+      <c r="D83" s="37" t="n">
+        <v>108.775</v>
+      </c>
+      <c r="E83" s="38" t="n">
+        <v>44.442</v>
+      </c>
+      <c r="F83" s="39" t="n">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="35" t="inlineStr">
+        <is>
+          <t>1+975</t>
+        </is>
+      </c>
+      <c r="B84" s="36" t="n">
+        <v>840801.0870000001</v>
+      </c>
+      <c r="C84" s="36" t="n">
+        <v>6518211.816</v>
+      </c>
+      <c r="D84" s="37" t="n">
+        <v>108.812</v>
+      </c>
+      <c r="E84" s="38" t="n">
+        <v>44.3696</v>
+      </c>
+      <c r="F84" s="39" t="n">
+        <v>1975</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="30" t="inlineStr">
+        <is>
+          <t>2+000</t>
+        </is>
+      </c>
+      <c r="B85" s="31" t="n">
+        <v>840816.716</v>
+      </c>
+      <c r="C85" s="31" t="n">
+        <v>6518231.497</v>
+      </c>
+      <c r="D85" s="32" t="n">
+        <v>108.85</v>
+      </c>
+      <c r="E85" s="33" t="n">
+        <v>44.2954</v>
+      </c>
+      <c r="F85" s="34" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="35" t="inlineStr">
+        <is>
+          <t>2+025</t>
+        </is>
+      </c>
+      <c r="B86" s="36" t="n">
+        <v>840832.252</v>
+      </c>
+      <c r="C86" s="36" t="n">
+        <v>6518251.265</v>
+      </c>
+      <c r="D86" s="37" t="n">
+        <v>108.887</v>
+      </c>
+      <c r="E86" s="38" t="n">
+        <v>44.2194</v>
+      </c>
+      <c r="F86" s="39" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="35" t="inlineStr">
+        <is>
+          <t>2+050</t>
+        </is>
+      </c>
+      <c r="B87" s="36" t="n">
+        <v>840847.6949999999</v>
+      </c>
+      <c r="C87" s="36" t="n">
+        <v>6518271.118</v>
+      </c>
+      <c r="D87" s="37" t="n">
+        <v>108.925</v>
+      </c>
+      <c r="E87" s="38" t="n">
+        <v>44.1418</v>
+      </c>
+      <c r="F87" s="39" t="n">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="35" t="inlineStr">
+        <is>
+          <t>2+075</t>
+        </is>
+      </c>
+      <c r="B88" s="36" t="n">
+        <v>840863.045</v>
+      </c>
+      <c r="C88" s="36" t="n">
+        <v>6518291.056</v>
+      </c>
+      <c r="D88" s="37" t="n">
+        <v>108.962</v>
+      </c>
+      <c r="E88" s="38" t="n">
+        <v>44.0625</v>
+      </c>
+      <c r="F88" s="39" t="n">
+        <v>2075</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="30" t="inlineStr">
+        <is>
+          <t>2+100</t>
+        </is>
+      </c>
+      <c r="B89" s="31" t="n">
+        <v>840878.302</v>
+      </c>
+      <c r="C89" s="31" t="n">
+        <v>6518311.078</v>
+      </c>
+      <c r="D89" s="32" t="n">
+        <v>109</v>
+      </c>
+      <c r="E89" s="33" t="n">
+        <v>43.9818</v>
+      </c>
+      <c r="F89" s="34" t="n">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="35" t="inlineStr">
+        <is>
+          <t>2+125</t>
+        </is>
+      </c>
+      <c r="B90" s="36" t="n">
+        <v>840893.466</v>
+      </c>
+      <c r="C90" s="36" t="n">
+        <v>6518331.183</v>
+      </c>
+      <c r="D90" s="37" t="n">
+        <v>109.037</v>
+      </c>
+      <c r="E90" s="38" t="n">
+        <v>43.8995</v>
+      </c>
+      <c r="F90" s="39" t="n">
+        <v>2125</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="35" t="inlineStr">
+        <is>
+          <t>2+150</t>
+        </is>
+      </c>
+      <c r="B91" s="36" t="n">
+        <v>840908.54</v>
+      </c>
+      <c r="C91" s="36" t="n">
+        <v>6518351.37</v>
+      </c>
+      <c r="D91" s="37" t="n">
+        <v>109.075</v>
+      </c>
+      <c r="E91" s="38" t="n">
+        <v>43.8159</v>
+      </c>
+      <c r="F91" s="39" t="n">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="35" t="inlineStr">
+        <is>
+          <t>2+175</t>
+        </is>
+      </c>
+      <c r="B92" s="36" t="n">
+        <v>840923.522</v>
+      </c>
+      <c r="C92" s="36" t="n">
+        <v>6518371.639</v>
+      </c>
+      <c r="D92" s="37" t="n">
+        <v>109.112</v>
+      </c>
+      <c r="E92" s="38" t="n">
+        <v>43.7311</v>
+      </c>
+      <c r="F92" s="39" t="n">
+        <v>2175</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="30" t="inlineStr">
+        <is>
+          <t>2+200</t>
+        </is>
+      </c>
+      <c r="B93" s="31" t="n">
+        <v>840938.4129999999</v>
+      </c>
+      <c r="C93" s="31" t="n">
+        <v>6518391.986</v>
+      </c>
+      <c r="D93" s="32" t="n">
+        <v>109.15</v>
+      </c>
+      <c r="E93" s="33" t="n">
+        <v>43.645</v>
+      </c>
+      <c r="F93" s="34" t="n">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="35" t="inlineStr">
+        <is>
+          <t>2+225</t>
+        </is>
+      </c>
+      <c r="B94" s="36" t="n">
+        <v>840953.216</v>
+      </c>
+      <c r="C94" s="36" t="n">
+        <v>6518412.412</v>
+      </c>
+      <c r="D94" s="37" t="n">
+        <v>109.188</v>
+      </c>
+      <c r="E94" s="38" t="n">
+        <v>43.5578</v>
+      </c>
+      <c r="F94" s="39" t="n">
+        <v>2225</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="35" t="inlineStr">
+        <is>
+          <t>2+250</t>
+        </is>
+      </c>
+      <c r="B95" s="36" t="n">
+        <v>840967.9300000001</v>
+      </c>
+      <c r="C95" s="36" t="n">
+        <v>6518432.915</v>
+      </c>
+      <c r="D95" s="37" t="n">
+        <v>109.225</v>
+      </c>
+      <c r="E95" s="38" t="n">
+        <v>43.4696</v>
+      </c>
+      <c r="F95" s="39" t="n">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="35" t="inlineStr">
+        <is>
+          <t>2+275</t>
+        </is>
+      </c>
+      <c r="B96" s="36" t="n">
+        <v>840982.558</v>
+      </c>
+      <c r="C96" s="36" t="n">
+        <v>6518453.493</v>
+      </c>
+      <c r="D96" s="37" t="n">
+        <v>109.262</v>
+      </c>
+      <c r="E96" s="38" t="n">
+        <v>43.3804</v>
+      </c>
+      <c r="F96" s="39" t="n">
+        <v>2275</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="30" t="inlineStr">
+        <is>
+          <t>2+300</t>
+        </is>
+      </c>
+      <c r="B97" s="31" t="n">
+        <v>840997.1</v>
+      </c>
+      <c r="C97" s="31" t="n">
+        <v>6518474.143</v>
+      </c>
+      <c r="D97" s="32" t="n">
+        <v>109.3</v>
+      </c>
+      <c r="E97" s="33" t="n">
+        <v>43.2903</v>
+      </c>
+      <c r="F97" s="34" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="35" t="inlineStr">
+        <is>
+          <t>2+325</t>
+        </is>
+      </c>
+      <c r="B98" s="36" t="n">
+        <v>841011.558</v>
+      </c>
+      <c r="C98" s="36" t="n">
+        <v>6518494.865</v>
+      </c>
+      <c r="D98" s="37" t="n">
+        <v>109.337</v>
+      </c>
+      <c r="E98" s="38" t="n">
+        <v>43.1995</v>
+      </c>
+      <c r="F98" s="39" t="n">
+        <v>2325</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="35" t="inlineStr">
+        <is>
+          <t>2+350</t>
+        </is>
+      </c>
+      <c r="B99" s="36" t="n">
+        <v>841025.934</v>
+      </c>
+      <c r="C99" s="36" t="n">
+        <v>6518515.656</v>
+      </c>
+      <c r="D99" s="37" t="n">
+        <v>109.375</v>
+      </c>
+      <c r="E99" s="38" t="n">
+        <v>43.108</v>
+      </c>
+      <c r="F99" s="39" t="n">
+        <v>2350</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="35" t="inlineStr">
+        <is>
+          <t>2+375</t>
+        </is>
+      </c>
+      <c r="B100" s="36" t="n">
+        <v>841040.23</v>
+      </c>
+      <c r="C100" s="36" t="n">
+        <v>6518536.514</v>
+      </c>
+      <c r="D100" s="37" t="n">
+        <v>109.412</v>
+      </c>
+      <c r="E100" s="38" t="n">
+        <v>43.016</v>
+      </c>
+      <c r="F100" s="39" t="n">
+        <v>2375</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="30" t="inlineStr">
+        <is>
+          <t>2+400</t>
+        </is>
+      </c>
+      <c r="B101" s="31" t="n">
+        <v>841054.447</v>
+      </c>
+      <c r="C101" s="31" t="n">
+        <v>6518557.437</v>
+      </c>
+      <c r="D101" s="32" t="n">
+        <v>109.45</v>
+      </c>
+      <c r="E101" s="33" t="n">
+        <v>42.9234</v>
+      </c>
+      <c r="F101" s="34" t="n">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="35" t="inlineStr">
+        <is>
+          <t>2+425</t>
+        </is>
+      </c>
+      <c r="B102" s="36" t="n">
+        <v>841068.588</v>
+      </c>
+      <c r="C102" s="36" t="n">
+        <v>6518578.422</v>
+      </c>
+      <c r="D102" s="37" t="n">
+        <v>109.487</v>
+      </c>
+      <c r="E102" s="38" t="n">
+        <v>42.8304</v>
+      </c>
+      <c r="F102" s="39" t="n">
+        <v>2425</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="35" t="inlineStr">
+        <is>
+          <t>2+450</t>
+        </is>
+      </c>
+      <c r="B103" s="36" t="n">
+        <v>841082.655</v>
+      </c>
+      <c r="C103" s="36" t="n">
+        <v>6518599.467</v>
+      </c>
+      <c r="D103" s="37" t="n">
+        <v>109.525</v>
+      </c>
+      <c r="E103" s="38" t="n">
+        <v>42.737</v>
+      </c>
+      <c r="F103" s="39" t="n">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="35" t="inlineStr">
+        <is>
+          <t>2+475</t>
+        </is>
+      </c>
+      <c r="B104" s="36" t="n">
+        <v>841096.65</v>
+      </c>
+      <c r="C104" s="36" t="n">
+        <v>6518620.569</v>
+      </c>
+      <c r="D104" s="37" t="n">
+        <v>109.562</v>
+      </c>
+      <c r="E104" s="38" t="n">
+        <v>42.6435</v>
+      </c>
+      <c r="F104" s="39" t="n">
+        <v>2475</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="30" t="inlineStr">
+        <is>
+          <t>2+500</t>
+        </is>
+      </c>
+      <c r="B105" s="31" t="n">
+        <v>841110.576</v>
+      </c>
+      <c r="C105" s="31" t="n">
+        <v>6518641.725</v>
+      </c>
+      <c r="D105" s="32" t="n">
+        <v>109.6</v>
+      </c>
+      <c r="E105" s="33" t="n">
+        <v>42.5498</v>
+      </c>
+      <c r="F105" s="34" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="35" t="inlineStr">
+        <is>
+          <t>2+525</t>
+        </is>
+      </c>
+      <c r="B106" s="36" t="n">
+        <v>841124.436</v>
+      </c>
+      <c r="C106" s="36" t="n">
+        <v>6518662.934</v>
+      </c>
+      <c r="D106" s="37" t="n">
+        <v>109.637</v>
+      </c>
+      <c r="E106" s="38" t="n">
+        <v>42.456</v>
+      </c>
+      <c r="F106" s="39" t="n">
+        <v>2525</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="35" t="inlineStr">
+        <is>
+          <t>2+550</t>
+        </is>
+      </c>
+      <c r="B107" s="36" t="n">
+        <v>841138.233</v>
+      </c>
+      <c r="C107" s="36" t="n">
+        <v>6518684.191</v>
+      </c>
+      <c r="D107" s="37" t="n">
+        <v>109.675</v>
+      </c>
+      <c r="E107" s="38" t="n">
+        <v>42.3623</v>
+      </c>
+      <c r="F107" s="39" t="n">
+        <v>2550</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="35" t="inlineStr">
+        <is>
+          <t>2+575</t>
+        </is>
+      </c>
+      <c r="B108" s="36" t="n">
+        <v>841151.968</v>
+      </c>
+      <c r="C108" s="36" t="n">
+        <v>6518705.495</v>
+      </c>
+      <c r="D108" s="37" t="n">
+        <v>109.712</v>
+      </c>
+      <c r="E108" s="38" t="n">
+        <v>42.2688</v>
+      </c>
+      <c r="F108" s="39" t="n">
+        <v>2575</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="30" t="inlineStr">
+        <is>
+          <t>2+600</t>
+        </is>
+      </c>
+      <c r="B109" s="31" t="n">
+        <v>841165.647</v>
+      </c>
+      <c r="C109" s="31" t="n">
+        <v>6518726.841</v>
+      </c>
+      <c r="D109" s="32" t="n">
+        <v>109.75</v>
+      </c>
+      <c r="E109" s="33" t="n">
+        <v>42.1754</v>
+      </c>
+      <c r="F109" s="34" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="35" t="inlineStr">
+        <is>
+          <t>2+625</t>
+        </is>
+      </c>
+      <c r="B110" s="36" t="n">
+        <v>841179.2709999999</v>
+      </c>
+      <c r="C110" s="36" t="n">
+        <v>6518748.227</v>
+      </c>
+      <c r="D110" s="37" t="n">
+        <v>109.787</v>
+      </c>
+      <c r="E110" s="38" t="n">
+        <v>42.0824</v>
+      </c>
+      <c r="F110" s="39" t="n">
+        <v>2625</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="35" t="inlineStr">
+        <is>
+          <t>2+650</t>
+        </is>
+      </c>
+      <c r="B111" s="36" t="n">
+        <v>841192.844</v>
+      </c>
+      <c r="C111" s="36" t="n">
+        <v>6518769.65</v>
+      </c>
+      <c r="D111" s="37" t="n">
+        <v>109.825</v>
+      </c>
+      <c r="E111" s="38" t="n">
+        <v>41.9898</v>
+      </c>
+      <c r="F111" s="39" t="n">
+        <v>2650</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="35" t="inlineStr">
+        <is>
+          <t>2+675</t>
+        </is>
+      </c>
+      <c r="B112" s="36" t="n">
+        <v>841206.37</v>
+      </c>
+      <c r="C112" s="36" t="n">
+        <v>6518791.107</v>
+      </c>
+      <c r="D112" s="37" t="n">
+        <v>109.862</v>
+      </c>
+      <c r="E112" s="38" t="n">
+        <v>41.8977</v>
+      </c>
+      <c r="F112" s="39" t="n">
+        <v>2675</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="30" t="inlineStr">
+        <is>
+          <t>2+700</t>
+        </is>
+      </c>
+      <c r="B113" s="31" t="n">
+        <v>841219.853</v>
+      </c>
+      <c r="C113" s="31" t="n">
+        <v>6518812.593</v>
+      </c>
+      <c r="D113" s="32" t="n">
+        <v>109.9</v>
+      </c>
+      <c r="E113" s="33" t="n">
+        <v>41.8061</v>
+      </c>
+      <c r="F113" s="34" t="n">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="35" t="inlineStr">
+        <is>
+          <t>2+725</t>
+        </is>
+      </c>
+      <c r="B114" s="36" t="n">
+        <v>841233.295</v>
+      </c>
+      <c r="C114" s="36" t="n">
+        <v>6518834.106</v>
+      </c>
+      <c r="D114" s="37" t="n">
+        <v>109.938</v>
+      </c>
+      <c r="E114" s="38" t="n">
+        <v>41.7153</v>
+      </c>
+      <c r="F114" s="39" t="n">
+        <v>2725</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="35" t="inlineStr">
+        <is>
+          <t>2+750</t>
+        </is>
+      </c>
+      <c r="B115" s="36" t="n">
+        <v>841246.701</v>
+      </c>
+      <c r="C115" s="36" t="n">
+        <v>6518855.642</v>
+      </c>
+      <c r="D115" s="37" t="n">
+        <v>109.975</v>
+      </c>
+      <c r="E115" s="38" t="n">
+        <v>41.6252</v>
+      </c>
+      <c r="F115" s="39" t="n">
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="35" t="inlineStr">
+        <is>
+          <t>2+775</t>
+        </is>
+      </c>
+      <c r="B116" s="36" t="n">
+        <v>841260.074</v>
+      </c>
+      <c r="C116" s="36" t="n">
+        <v>6518877.198</v>
+      </c>
+      <c r="D116" s="37" t="n">
+        <v>110.012</v>
+      </c>
+      <c r="E116" s="38" t="n">
+        <v>41.5359</v>
+      </c>
+      <c r="F116" s="39" t="n">
+        <v>2775</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="30" t="inlineStr">
+        <is>
+          <t>2+800</t>
+        </is>
+      </c>
+      <c r="B117" s="31" t="n">
+        <v>841273.419</v>
+      </c>
+      <c r="C117" s="31" t="n">
+        <v>6518898.77</v>
+      </c>
+      <c r="D117" s="32" t="n">
+        <v>110.05</v>
+      </c>
+      <c r="E117" s="33" t="n">
+        <v>41.4477</v>
+      </c>
+      <c r="F117" s="34" t="n">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="35" t="inlineStr">
+        <is>
+          <t>2+825</t>
+        </is>
+      </c>
+      <c r="B118" s="36" t="n">
+        <v>841286.74</v>
+      </c>
+      <c r="C118" s="36" t="n">
+        <v>6518920.355</v>
+      </c>
+      <c r="D118" s="37" t="n">
+        <v>110.087</v>
+      </c>
+      <c r="E118" s="38" t="n">
+        <v>41.3604</v>
+      </c>
+      <c r="F118" s="39" t="n">
+        <v>2825</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="35" t="inlineStr">
+        <is>
+          <t>2+850</t>
+        </is>
+      </c>
+      <c r="B119" s="36" t="n">
+        <v>841300.042</v>
+      </c>
+      <c r="C119" s="36" t="n">
+        <v>6518941.948</v>
+      </c>
+      <c r="D119" s="37" t="n">
+        <v>110.125</v>
+      </c>
+      <c r="E119" s="38" t="n">
+        <v>41.2742</v>
+      </c>
+      <c r="F119" s="39" t="n">
+        <v>2850</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="35" t="inlineStr">
+        <is>
+          <t>2+875</t>
+        </is>
+      </c>
+      <c r="B120" s="36" t="n">
+        <v>841313.327</v>
+      </c>
+      <c r="C120" s="36" t="n">
+        <v>6518963.547</v>
+      </c>
+      <c r="D120" s="37" t="n">
+        <v>110.162</v>
+      </c>
+      <c r="E120" s="38" t="n">
+        <v>41.1893</v>
+      </c>
+      <c r="F120" s="39" t="n">
+        <v>2875</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="30" t="inlineStr">
+        <is>
+          <t>2+900</t>
+        </is>
+      </c>
+      <c r="B121" s="31" t="n">
+        <v>841326.602</v>
+      </c>
+      <c r="C121" s="31" t="n">
+        <v>6518985.147</v>
+      </c>
+      <c r="D121" s="32" t="n">
+        <v>110.2</v>
+      </c>
+      <c r="E121" s="33" t="n">
+        <v>41.1056</v>
+      </c>
+      <c r="F121" s="34" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="35" t="inlineStr">
+        <is>
+          <t>2+925</t>
+        </is>
+      </c>
+      <c r="B122" s="36" t="n">
+        <v>841339.87</v>
+      </c>
+      <c r="C122" s="36" t="n">
+        <v>6519006.745</v>
+      </c>
+      <c r="D122" s="37" t="n">
+        <v>110.237</v>
+      </c>
+      <c r="E122" s="38" t="n">
+        <v>41.0233</v>
+      </c>
+      <c r="F122" s="39" t="n">
+        <v>2925</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="35" t="inlineStr">
+        <is>
+          <t>2+950</t>
+        </is>
+      </c>
+      <c r="B123" s="36" t="n">
+        <v>841353.1360000001</v>
+      </c>
+      <c r="C123" s="36" t="n">
+        <v>6519028.337</v>
+      </c>
+      <c r="D123" s="37" t="n">
+        <v>110.275</v>
+      </c>
+      <c r="E123" s="38" t="n">
+        <v>40.9424</v>
+      </c>
+      <c r="F123" s="39" t="n">
+        <v>2950</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="35" t="inlineStr">
+        <is>
+          <t>2+975</t>
+        </is>
+      </c>
+      <c r="B124" s="36" t="n">
+        <v>841366.404</v>
+      </c>
+      <c r="C124" s="36" t="n">
+        <v>6519049.919</v>
+      </c>
+      <c r="D124" s="37" t="n">
+        <v>110.312</v>
+      </c>
+      <c r="E124" s="38" t="n">
+        <v>40.8631</v>
+      </c>
+      <c r="F124" s="39" t="n">
+        <v>2975</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="30" t="inlineStr">
+        <is>
+          <t>3+000</t>
+        </is>
+      </c>
+      <c r="B125" s="31" t="n">
+        <v>841379.6800000001</v>
+      </c>
+      <c r="C125" s="31" t="n">
+        <v>6519071.487</v>
+      </c>
+      <c r="D125" s="32" t="n">
+        <v>110.35</v>
+      </c>
+      <c r="E125" s="33" t="n">
+        <v>40.7853</v>
+      </c>
+      <c r="F125" s="34" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="127" ht="30" customHeight="1">
+      <c r="A127" s="40" t="inlineStr">
+        <is>
+          <t>IMPORTANT : Ces coordonnées sont générées automatiquement (projet démo). Remplacer par les coordonnées réelles issues du levé topographique ou du GPS.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:F125"/>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A127:F127"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>DISTANCES TRANSVERSALES / AXE — Route Nationale 2x2 voies TPC — 3 km</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="42" t="inlineStr">
+        <is>
+          <t>SECTION EN TRAVERS TYPE — Vue schématique (de gauche à droite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="14" customHeight="1">
+      <c r="A3" s="43" t="inlineStr"/>
+    </row>
+    <row r="4" ht="14" customHeight="1">
+      <c r="A4" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ← GAUCHE (distances négatives)        AXE        DROITE (distances positives) →</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="14" customHeight="1">
+      <c r="A5" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ─────────────────────────────────────── 0 ────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="A6" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Bord_Prop_G ... Canal_G ... Bord_Chaussee_G   |   Bord_Chaussee_D ... Canal_D ... Bord_Prop_D</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="44" t="inlineStr">
+        <is>
+          <t>Élément</t>
+        </is>
+      </c>
+      <c r="B7" s="44" t="inlineStr">
+        <is>
+          <t>Distance / axe (m)</t>
+        </is>
+      </c>
+      <c r="C7" s="44" t="inlineStr">
+        <is>
+          <t>Côté</t>
+        </is>
+      </c>
+      <c r="D7" s="44" t="inlineStr">
+        <is>
+          <t>Colonne cote référence</t>
+        </is>
+      </c>
+      <c r="E7" s="44" t="inlineStr">
+        <is>
+          <t>Onglet source</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="45" t="inlineStr">
+        <is>
+          <t>AXE</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="47" t="inlineStr">
+        <is>
+          <t>Axe</t>
+        </is>
+      </c>
+      <c r="D8" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="48" t="inlineStr">
+        <is>
+          <t>TPC_Gauche</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="C9" s="48" t="inlineStr">
+        <is>
+          <t>Gauche</t>
+        </is>
+      </c>
+      <c r="D9" s="48" t="inlineStr">
+        <is>
+          <t>AXE_G</t>
+        </is>
+      </c>
+      <c r="E9" s="48" t="inlineStr">
+        <is>
+          <t>Cote_Gauche</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="50" t="inlineStr">
+        <is>
+          <t>TPC_Droit</t>
+        </is>
+      </c>
+      <c r="B10" s="51" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C10" s="50" t="inlineStr">
+        <is>
+          <t>Droit</t>
+        </is>
+      </c>
+      <c r="D10" s="50" t="inlineStr">
+        <is>
+          <t>AXE_D</t>
+        </is>
+      </c>
+      <c r="E10" s="50" t="inlineStr">
+        <is>
+          <t>Cote_Droit</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="48" t="inlineStr">
+        <is>
+          <t>Bord_Chaussee_G</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="C11" s="48" t="inlineStr">
+        <is>
+          <t>Gauche</t>
+        </is>
+      </c>
+      <c r="D11" s="48" t="inlineStr">
+        <is>
+          <t>Tablier_Fini_G</t>
+        </is>
+      </c>
+      <c r="E11" s="48" t="inlineStr">
+        <is>
+          <t>Cote_Gauche</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="50" t="inlineStr">
+        <is>
+          <t>Bord_Chaussee_D</t>
+        </is>
+      </c>
+      <c r="B12" s="51" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C12" s="50" t="inlineStr">
+        <is>
+          <t>Droit</t>
+        </is>
+      </c>
+      <c r="D12" s="50" t="inlineStr">
+        <is>
+          <t>Tablier_Fini_D</t>
+        </is>
+      </c>
+      <c r="E12" s="50" t="inlineStr">
+        <is>
+          <t>Cote_Droit</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>Canal_G (100x100)</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="C13" s="48" t="inlineStr">
+        <is>
+          <t>Gauche</t>
+        </is>
+      </c>
+      <c r="D13" s="48" t="inlineStr">
+        <is>
+          <t>Tablier_Fini_G</t>
+        </is>
+      </c>
+      <c r="E13" s="48" t="inlineStr">
+        <is>
+          <t>Cote_Gauche</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="50" t="inlineStr">
+        <is>
+          <t>Canal_D (60x60)</t>
+        </is>
+      </c>
+      <c r="B14" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="C14" s="50" t="inlineStr">
+        <is>
+          <t>Droit</t>
+        </is>
+      </c>
+      <c r="D14" s="50" t="inlineStr">
+        <is>
+          <t>Tablier_Fini_D</t>
+        </is>
+      </c>
+      <c r="E14" s="50" t="inlineStr">
+        <is>
+          <t>Cote_Droit</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="48" t="inlineStr">
+        <is>
+          <t>Accotement_G</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="C15" s="48" t="inlineStr">
+        <is>
+          <t>Gauche</t>
+        </is>
+      </c>
+      <c r="D15" s="48" t="inlineStr">
+        <is>
+          <t>Bord_Propriete_G</t>
+        </is>
+      </c>
+      <c r="E15" s="48" t="inlineStr">
+        <is>
+          <t>Cote_Gauche</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="50" t="inlineStr">
+        <is>
+          <t>Accotement_D</t>
+        </is>
+      </c>
+      <c r="B16" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="C16" s="50" t="inlineStr">
+        <is>
+          <t>Droit</t>
+        </is>
+      </c>
+      <c r="D16" s="50" t="inlineStr">
+        <is>
+          <t>Bord_Propriete_D</t>
+        </is>
+      </c>
+      <c r="E16" s="50" t="inlineStr">
+        <is>
+          <t>Cote_Droit</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="48" t="inlineStr">
+        <is>
+          <t>Bord_Propriete_G</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="n">
+        <v>-12</v>
+      </c>
+      <c r="C17" s="48" t="inlineStr">
+        <is>
+          <t>Gauche</t>
+        </is>
+      </c>
+      <c r="D17" s="48" t="inlineStr">
+        <is>
+          <t>Bord_Propriete_G</t>
+        </is>
+      </c>
+      <c r="E17" s="48" t="inlineStr">
+        <is>
+          <t>Cote_Gauche</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="50" t="inlineStr">
+        <is>
+          <t>Bord_Propriete_D</t>
+        </is>
+      </c>
+      <c r="B18" s="51" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C18" s="50" t="inlineStr">
+        <is>
+          <t>Droit</t>
+        </is>
+      </c>
+      <c r="D18" s="50" t="inlineStr">
+        <is>
+          <t>Bord_Propriete_D</t>
+        </is>
+      </c>
+      <c r="E18" s="50" t="inlineStr">
+        <is>
+          <t>Cote_Droit</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="52" t="inlineStr">
+        <is>
+          <t>UTILISATION :
+• La colonne 'Distance / axe' donne la position transversale de chaque élément (- = gauche, + = droite).
+• Combinée aux coordonnées XY de PK_Coordonnees, elle permet de calculer la position GPS de chaque élément via : X_elem = X_axe + dist × sin(gisement + 90°) / Y_elem = Y_axe + dist × cos(gisement + 90°).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1"/>
+    <row r="22" ht="18" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A20:E22"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>